<commit_message>
sync kpi_logic and update goal ratings
</commit_message>
<xml_diff>
--- a/data/supplementary_kpis.xlsx
+++ b/data/supplementary_kpis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sap-my.sharepoint.com/personal/shameer_thajudeen_sap_com/Documents/Desktop/EC BLR 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADD6EA0D-91EB-4192-B0C0-895C574251F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3B965AF-8398-4BD3-A1A0-BF45C2CD2573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
     <t>nCES</t>
   </si>
   <si>
-    <t>Surveys</t>
+    <t># Top 2 Box Surveys</t>
   </si>
   <si>
     <t>KCS Focus</t>
@@ -1797,6 +1797,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{0cf7ac0a-4681-4823-ab0b-04ef02c5f873}" enabled="1" method="Standard" siteId="{42f7676c-f455-423c-82f6-dc2d99791af7}" contentBits="0" removed="0"/>
+  <clbl:label id="{0cf7ac0a-4681-4823-ab0b-04ef02c5f873}" enabled="1" method="Standard" siteId="{42f7676c-f455-423c-82f6-dc2d99791af7}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>